<commit_message>
feat: support custom directories and nested basic materials
</commit_message>
<xml_diff>
--- a/examples/demo-labor-dispute/1-林晚晴等VS沪江优配等-劳动争议/整理结果/案件材料汇总.xlsx
+++ b/examples/demo-labor-dispute/1-林晚晴等VS沪江优配等-劳动争议/整理结果/案件材料汇总.xlsx
@@ -1067,7 +1067,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/03 加班与沟通</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/02 工资付款与扣款</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/04 事故医疗与现场</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/01 合同协议</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/02 工资付款与扣款</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/02 工资付款与扣款</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/01 合同协议</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/04 事故医疗与现场</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/02 工资付款与扣款</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/04 事故医疗与现场</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
+          <t>002 基础资料/02 工资付款与扣款</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">

</xml_diff>